<commit_message>
Refactor program construction and gameloop
</commit_message>
<xml_diff>
--- a/note/color.xlsx
+++ b/note/color.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdme\git\myrmidon\note\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44F7E48-72E8-464C-89F4-7CFFAD0BD743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82722557-6EF8-4751-9C67-8184162350D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{4E1ADB55-CAD3-4A88-8BA6-1F73A783538E}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4E1ADB55-CAD3-4A88-8BA6-1F73A783538E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -219,6 +219,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -365,11 +369,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -435,8 +440,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -770,14 +777,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A548D68-F811-4DF9-9498-4CD29637B929}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.5" customWidth="1"/>
     <col min="8" max="8" width="4.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -811,7 +818,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -838,22 +845,34 @@
       </c>
       <c r="H2" s="22"/>
       <c r="I2" s="22">
-        <f>(1-E2-L2)/(1-L2)</f>
+        <f t="shared" ref="I2:I7" si="0">(1-E2-L2)/(1-L2)</f>
         <v>0</v>
       </c>
       <c r="J2" s="22">
-        <f t="shared" ref="J2:J7" si="0">(1-F2-L2)/(1-L2)</f>
+        <f t="shared" ref="J2:J7" si="1">(1-F2-L2)/(1-L2)</f>
         <v>0.55421686746987942</v>
       </c>
       <c r="K2" s="22">
         <v>0.72</v>
       </c>
       <c r="L2" s="22">
-        <f>1-MAX(E2:G2)</f>
+        <f t="shared" ref="L2:L7" si="2">1-MAX(E2:G2)</f>
         <v>0.34901960784313724</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N2" s="23">
+        <f>HEX2DEC(RIGHT(LEFT(C2,3),2))</f>
+        <v>166</v>
+      </c>
+      <c r="O2" s="23">
+        <f>HEX2DEC(RIGHT(LEFT(C2,5),2))</f>
+        <v>74</v>
+      </c>
+      <c r="P2" s="23">
+        <f>HEX2DEC(RIGHT(C2,2))</f>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
@@ -867,35 +886,47 @@
         <v>6</v>
       </c>
       <c r="E3" s="22">
-        <f t="shared" ref="E3:E21" si="1">HEX2DEC(RIGHT(LEFT(C3,3),2))/255</f>
+        <f t="shared" ref="E3:E21" si="3">HEX2DEC(RIGHT(LEFT(C3,3),2))/255</f>
         <v>0.84313725490196079</v>
       </c>
       <c r="F3" s="22">
-        <f t="shared" ref="F3:F21" si="2">HEX2DEC(RIGHT(LEFT(C3,5),2))/255</f>
+        <f t="shared" ref="F3:F21" si="4">HEX2DEC(RIGHT(LEFT(C3,5),2))/255</f>
         <v>0.25882352941176473</v>
       </c>
       <c r="G3" s="22">
-        <f t="shared" ref="G3:G21" si="3">HEX2DEC(RIGHT(C3,2))/255</f>
+        <f t="shared" ref="G3:G21" si="5">HEX2DEC(RIGHT(C3,2))/255</f>
         <v>0</v>
       </c>
       <c r="H3" s="22"/>
       <c r="I3" s="22">
-        <f>(1-E3-L3)/(1-L3)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J3" s="22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.69302325581395352</v>
       </c>
       <c r="K3" s="22">
         <v>1</v>
       </c>
       <c r="L3" s="22">
-        <f>1-MAX(E3:G3)</f>
+        <f t="shared" si="2"/>
         <v>0.15686274509803921</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N3" s="23">
+        <f t="shared" ref="N3:N21" si="6">HEX2DEC(RIGHT(LEFT(C3,3),2))</f>
+        <v>215</v>
+      </c>
+      <c r="O3" s="23">
+        <f t="shared" ref="O3:O21" si="7">HEX2DEC(RIGHT(LEFT(C3,5),2))</f>
+        <v>66</v>
+      </c>
+      <c r="P3" s="23">
+        <f t="shared" ref="P3:P21" si="8">HEX2DEC(RIGHT(C3,2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -909,36 +940,48 @@
         <v>6</v>
       </c>
       <c r="E4" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F4" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.58039215686274515</v>
       </c>
       <c r="G4" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.1764705882352941E-2</v>
       </c>
       <c r="H4" s="22"/>
       <c r="I4" s="22">
-        <f>(1-E4-L4)/(1-L4)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J4" s="22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K4" s="22">
-        <f t="shared" ref="K4:K7" si="4">(1-G4-L4)/(1-L4)</f>
+        <f t="shared" ref="K4:K7" si="9">(1-G4-L4)/(1-L4)</f>
         <v>0.97972972972972983</v>
       </c>
       <c r="L4" s="22">
-        <f>1-MAX(E4:G4)</f>
+        <f t="shared" si="2"/>
         <v>0.41960784313725485</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N4" s="23">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="O4" s="23">
+        <f t="shared" si="7"/>
+        <v>148</v>
+      </c>
+      <c r="P4" s="23">
+        <f t="shared" si="8"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>25</v>
       </c>
@@ -952,36 +995,48 @@
         <v>6</v>
       </c>
       <c r="E5" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F5" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.7686274509803922</v>
       </c>
       <c r="G5" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.12549019607843137</v>
       </c>
       <c r="H5" s="22"/>
       <c r="I5" s="22">
-        <f>(1-E5-L5)/(1-L5)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J5" s="22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K5" s="22">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.83673469387755106</v>
       </c>
       <c r="L5" s="22">
-        <f>1-MAX(E5:G5)</f>
+        <f t="shared" si="2"/>
         <v>0.2313725490196078</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N5" s="23">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="23">
+        <f t="shared" si="7"/>
+        <v>196</v>
+      </c>
+      <c r="P5" s="23">
+        <f t="shared" si="8"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -995,36 +1050,48 @@
         <v>6</v>
       </c>
       <c r="E6" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F6" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.28235294117647058</v>
       </c>
       <c r="G6" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.74117647058823533</v>
       </c>
       <c r="H6" s="22"/>
       <c r="I6" s="22">
-        <f>(1-E6-L6)/(1-L6)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J6" s="22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.61904761904761907</v>
       </c>
       <c r="K6" s="22">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="L6" s="22">
-        <f>1-MAX(E6:G6)</f>
+        <f t="shared" si="2"/>
         <v>0.25882352941176467</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N6" s="23">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="O6" s="23">
+        <f t="shared" si="7"/>
+        <v>72</v>
+      </c>
+      <c r="P6" s="23">
+        <f t="shared" si="8"/>
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
         <v>31</v>
       </c>
@@ -1038,36 +1105,48 @@
         <v>6</v>
       </c>
       <c r="E7" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F7" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.58823529411764708</v>
       </c>
       <c r="G7" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H7" s="22"/>
       <c r="I7" s="22">
-        <f>(1-E7-L7)/(1-L7)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="J7" s="22">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.41176470588235292</v>
       </c>
       <c r="K7" s="22">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="L7" s="22">
-        <f>1-MAX(E7:G7)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N7" s="23">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="23">
+        <f t="shared" si="7"/>
+        <v>150</v>
+      </c>
+      <c r="P7" s="23">
+        <f t="shared" si="8"/>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1080,8 +1159,11 @@
       <c r="J8" s="22"/>
       <c r="K8" s="22"/>
       <c r="L8" s="22"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="23"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
@@ -1095,35 +1177,47 @@
         <v>6</v>
       </c>
       <c r="E9" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.25098039215686274</v>
       </c>
       <c r="F9" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.64313725490196083</v>
       </c>
       <c r="G9" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.72549019607843135</v>
       </c>
       <c r="H9" s="22"/>
       <c r="I9" s="22">
-        <f>(1-E9-L9)/(1-L9)</f>
+        <f t="shared" ref="I9:I16" si="10">(1-E9-L9)/(1-L9)</f>
         <v>0.65405405405405403</v>
       </c>
       <c r="J9" s="22">
-        <f t="shared" ref="J9:J16" si="5">(1-F9-L9)/(1-L9)</f>
+        <f t="shared" ref="J9:J16" si="11">(1-F9-L9)/(1-L9)</f>
         <v>0.11351351351351342</v>
       </c>
       <c r="K9" s="22">
         <v>0</v>
       </c>
       <c r="L9" s="22">
-        <f>1-MAX(E9:G9)</f>
+        <f t="shared" ref="L9:L16" si="12">1-MAX(E9:G9)</f>
         <v>0.27450980392156865</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N9" s="23">
+        <f t="shared" si="6"/>
+        <v>64</v>
+      </c>
+      <c r="O9" s="23">
+        <f t="shared" si="7"/>
+        <v>164</v>
+      </c>
+      <c r="P9" s="23">
+        <f t="shared" si="8"/>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
         <v>37</v>
       </c>
@@ -1137,35 +1231,47 @@
         <v>6</v>
       </c>
       <c r="E10" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.46666666666666667</v>
       </c>
       <c r="F10" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.74901960784313726</v>
       </c>
       <c r="G10" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.81176470588235294</v>
       </c>
       <c r="H10" s="22"/>
       <c r="I10" s="22">
-        <f>(1-E10-L10)/(1-L10)</f>
+        <f t="shared" si="10"/>
         <v>0.4251207729468599</v>
       </c>
       <c r="J10" s="22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>7.7294685990338161E-2</v>
       </c>
       <c r="K10" s="22">
         <v>0</v>
       </c>
       <c r="L10" s="22">
-        <f>1-MAX(E10:G10)</f>
+        <f t="shared" si="12"/>
         <v>0.18823529411764706</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N10" s="23">
+        <f t="shared" si="6"/>
+        <v>119</v>
+      </c>
+      <c r="O10" s="23">
+        <f t="shared" si="7"/>
+        <v>191</v>
+      </c>
+      <c r="P10" s="23">
+        <f t="shared" si="8"/>
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>40</v>
       </c>
@@ -1179,35 +1285,47 @@
         <v>6</v>
       </c>
       <c r="E11" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.69411764705882351</v>
       </c>
       <c r="F11" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.32941176470588235</v>
       </c>
       <c r="G11" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.81176470588235294</v>
       </c>
       <c r="H11" s="22"/>
       <c r="I11" s="22">
-        <f>(1-E11-L11)/(1-L11)</f>
+        <f t="shared" si="10"/>
         <v>0.14492753623188409</v>
       </c>
       <c r="J11" s="22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>0.59420289855072472</v>
       </c>
       <c r="K11" s="22">
         <v>0</v>
       </c>
       <c r="L11" s="22">
-        <f>1-MAX(E11:G11)</f>
+        <f t="shared" si="12"/>
         <v>0.18823529411764706</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N11" s="23">
+        <f t="shared" si="6"/>
+        <v>177</v>
+      </c>
+      <c r="O11" s="23">
+        <f t="shared" si="7"/>
+        <v>84</v>
+      </c>
+      <c r="P11" s="23">
+        <f t="shared" si="8"/>
+        <v>207</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
         <v>43</v>
       </c>
@@ -1221,35 +1339,47 @@
         <v>6</v>
       </c>
       <c r="E12" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.85490196078431369</v>
       </c>
       <c r="F12" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.35686274509803922</v>
       </c>
       <c r="G12" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.83921568627450982</v>
       </c>
       <c r="H12" s="22"/>
       <c r="I12" s="22">
-        <f>(1-E12-L12)/(1-L12)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J12" s="22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>0.58256880733944949</v>
       </c>
       <c r="K12" s="22">
         <v>0.02</v>
       </c>
       <c r="L12" s="22">
-        <f>1-MAX(E12:G12)</f>
+        <f t="shared" si="12"/>
         <v>0.14509803921568631</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N12" s="23">
+        <f t="shared" si="6"/>
+        <v>218</v>
+      </c>
+      <c r="O12" s="23">
+        <f t="shared" si="7"/>
+        <v>91</v>
+      </c>
+      <c r="P12" s="23">
+        <f t="shared" si="8"/>
+        <v>214</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>51</v>
       </c>
@@ -1263,35 +1393,47 @@
         <v>6</v>
       </c>
       <c r="E13" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.69411764705882351</v>
       </c>
       <c r="F13" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.78823529411764703</v>
       </c>
       <c r="G13" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.76470588235294112</v>
       </c>
       <c r="H13" s="22"/>
       <c r="I13" s="22">
-        <f>(1-E13-L13)/(1-L13)</f>
+        <f t="shared" si="10"/>
         <v>0.11940298507462686</v>
       </c>
       <c r="J13" s="22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="K13" s="22">
         <v>0.03</v>
       </c>
       <c r="L13" s="22">
-        <f>1-MAX(E13:G13)</f>
+        <f t="shared" si="12"/>
         <v>0.21176470588235297</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N13" s="23">
+        <f t="shared" si="6"/>
+        <v>177</v>
+      </c>
+      <c r="O13" s="23">
+        <f t="shared" si="7"/>
+        <v>201</v>
+      </c>
+      <c r="P13" s="23">
+        <f t="shared" si="8"/>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
         <v>54</v>
       </c>
@@ -1305,35 +1447,47 @@
         <v>6</v>
       </c>
       <c r="E14" s="22">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F14" s="22">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="G14" s="22">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
+      <c r="F14" s="22">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="G14" s="22">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
       <c r="H14" s="22"/>
       <c r="I14" s="22">
-        <f>(1-E14-L14)/(1-L14)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J14" s="22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="K14" s="22">
         <v>0</v>
       </c>
       <c r="L14" s="22">
-        <f>1-MAX(E14:G14)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="N14" s="23">
+        <f t="shared" si="6"/>
+        <v>255</v>
+      </c>
+      <c r="O14" s="23">
+        <f t="shared" si="7"/>
+        <v>255</v>
+      </c>
+      <c r="P14" s="23">
+        <f t="shared" si="8"/>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>46</v>
       </c>
@@ -1345,35 +1499,47 @@
         <v>6</v>
       </c>
       <c r="E15" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>5.8823529411764705E-2</v>
       </c>
       <c r="F15" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.23137254901960785</v>
       </c>
       <c r="G15" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.22745098039215686</v>
       </c>
       <c r="H15" s="22"/>
       <c r="I15" s="22">
-        <f>(1-E15-L15)/(1-L15)</f>
+        <f t="shared" si="10"/>
         <v>0.74576271186440679</v>
       </c>
       <c r="J15" s="22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="K15" s="22">
         <v>0</v>
       </c>
       <c r="L15" s="22">
-        <f>1-MAX(E15:G15)</f>
+        <f t="shared" si="12"/>
         <v>0.76862745098039209</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N15" s="23">
+        <f t="shared" si="6"/>
+        <v>15</v>
+      </c>
+      <c r="O15" s="23">
+        <f t="shared" si="7"/>
+        <v>59</v>
+      </c>
+      <c r="P15" s="23">
+        <f t="shared" si="8"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
         <v>48</v>
       </c>
@@ -1387,35 +1553,47 @@
         <v>6</v>
       </c>
       <c r="E16" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>8.2352941176470587E-2</v>
       </c>
       <c r="F16" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.32549019607843138</v>
       </c>
       <c r="G16" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.32156862745098042</v>
       </c>
       <c r="H16" s="22"/>
       <c r="I16" s="22">
-        <f>(1-E16-L16)/(1-L16)</f>
+        <f t="shared" si="10"/>
         <v>0.74698795180722877</v>
       </c>
       <c r="J16" s="22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="K16" s="22">
         <v>0.01</v>
       </c>
       <c r="L16" s="22">
-        <f>1-MAX(E16:G16)</f>
+        <f t="shared" si="12"/>
         <v>0.67450980392156867</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N16" s="23">
+        <f t="shared" si="6"/>
+        <v>21</v>
+      </c>
+      <c r="O16" s="23">
+        <f t="shared" si="7"/>
+        <v>83</v>
+      </c>
+      <c r="P16" s="23">
+        <f t="shared" si="8"/>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1428,8 +1606,20 @@
       <c r="J17" s="22"/>
       <c r="K17" s="22"/>
       <c r="L17" s="22"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N17" s="23">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="O17" s="23">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="P17" s="23">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>10</v>
       </c>
@@ -1443,15 +1633,15 @@
         <v>6</v>
       </c>
       <c r="E18" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.94509803921568625</v>
       </c>
       <c r="F18" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.37254901960784315</v>
       </c>
       <c r="G18" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.13333333333333333</v>
       </c>
       <c r="H18" s="22"/>
@@ -1471,8 +1661,20 @@
         <f>1-MAX(E18:G18)</f>
         <v>5.4901960784313752E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N18" s="23">
+        <f t="shared" si="6"/>
+        <v>241</v>
+      </c>
+      <c r="O18" s="23">
+        <f t="shared" si="7"/>
+        <v>95</v>
+      </c>
+      <c r="P18" s="23">
+        <f t="shared" si="8"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>13</v>
       </c>
@@ -1486,15 +1688,15 @@
         <v>6</v>
       </c>
       <c r="E19" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.9137254901960784</v>
       </c>
       <c r="F19" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.62352941176470589</v>
       </c>
       <c r="G19" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.2745098039215685E-2</v>
       </c>
       <c r="H19" s="22"/>
@@ -1503,19 +1705,31 @@
         <v>0</v>
       </c>
       <c r="J19" s="22">
-        <f t="shared" ref="J19:J21" si="6">(1-F19-L19)/(1-L19)</f>
+        <f t="shared" ref="J19:J21" si="13">(1-F19-L19)/(1-L19)</f>
         <v>0.31759656652360513</v>
       </c>
       <c r="K19" s="22">
-        <f t="shared" ref="K19:K21" si="7">(1-G19-L19)/(1-L19)</f>
+        <f t="shared" ref="K19:K21" si="14">(1-G19-L19)/(1-L19)</f>
         <v>0.93133047210300424</v>
       </c>
       <c r="L19" s="22">
         <f>1-MAX(E19:G19)</f>
         <v>8.6274509803921595E-2</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N19" s="23">
+        <f t="shared" si="6"/>
+        <v>233</v>
+      </c>
+      <c r="O19" s="23">
+        <f t="shared" si="7"/>
+        <v>159</v>
+      </c>
+      <c r="P19" s="23">
+        <f t="shared" si="8"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -1529,15 +1743,15 @@
         <v>6</v>
       </c>
       <c r="E20" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.59607843137254901</v>
       </c>
       <c r="F20" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.52941176470588236</v>
       </c>
       <c r="G20" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.37254901960784315</v>
       </c>
       <c r="H20" s="22"/>
@@ -1546,19 +1760,31 @@
         <v>0</v>
       </c>
       <c r="J20" s="22">
-        <f t="shared" si="6"/>
+        <f t="shared" si="13"/>
         <v>0.11184210526315787</v>
       </c>
       <c r="K20" s="22">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>0.375</v>
       </c>
       <c r="L20" s="22">
         <f>1-MAX(E20:G20)</f>
         <v>0.40392156862745099</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="N20" s="23">
+        <f t="shared" si="6"/>
+        <v>152</v>
+      </c>
+      <c r="O20" s="23">
+        <f t="shared" si="7"/>
+        <v>135</v>
+      </c>
+      <c r="P20" s="23">
+        <f t="shared" si="8"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -1572,15 +1798,15 @@
         <v>6</v>
       </c>
       <c r="E21" s="22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.81176470588235294</v>
       </c>
       <c r="F21" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.75294117647058822</v>
       </c>
       <c r="G21" s="22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.25490196078431371</v>
       </c>
       <c r="H21" s="22"/>
@@ -1589,19 +1815,31 @@
         <v>0</v>
       </c>
       <c r="J21" s="22">
-        <f t="shared" si="6"/>
+        <f t="shared" si="13"/>
         <v>7.2463768115942045E-2</v>
       </c>
       <c r="K21" s="22">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>0.68599033816425126</v>
       </c>
       <c r="L21" s="22">
         <f>1-MAX(E21:G21)</f>
         <v>0.18823529411764706</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="N21" s="23">
+        <f t="shared" si="6"/>
+        <v>207</v>
+      </c>
+      <c r="O21" s="23">
+        <f t="shared" si="7"/>
+        <v>192</v>
+      </c>
+      <c r="P21" s="23">
+        <f t="shared" si="8"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="C24" s="2" t="s">
         <v>57</v>
       </c>

</xml_diff>